<commit_message>
After D day (#1)
* D-Day code

Safety check, green LED, trigger

* Shooting data

Added some data in comment

* I2C and LED

I2C no longer need to be between 0-2;
LED less blinking

* Delay

Added delay at the start
</commit_message>
<xml_diff>
--- a/Budget.xlsx
+++ b/Budget.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hkustconnect-my.sharepoint.com/personal/tkzhang_connect_ust_hk/Documents/26 Spring/MECH3907/2026-MECH3907-Gp7-TTB-shooter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="348" documentId="11_C05832F84A9D4BDE4F2273C8C3656160CE96F8EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67ABB5CA-222B-4E9B-8A51-24014EC83669}"/>
+  <xr:revisionPtr revIDLastSave="395" documentId="11_C05832F84A9D4BDE4F2273C8C3656160CE96F8EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64ADBFEE-08AB-47F6-ADDB-8128FA49271E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="44">
   <si>
     <t>Item 
 no.</t>
@@ -110,10 +110,6 @@
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
-    <t>M from robotics team :&lt;</t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
     <t>Linear bearing</t>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
@@ -122,59 +118,11 @@
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
-    <t>SCSAW6</t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">https://item.taobao.com/item.htm?from=cart&amp;id=811026453751&amp;mi_id=0000_kb-1ZNX-l03ISmACZMSnVZf7Ow_MXV4ptcRVp0VqGk&amp;skuId=6153149310541&amp;spm=a1z0d.6639537%2F202410.item.d811026453751.3d385886TqyZCj&amp;upStreamPrice=155 </t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t>Can be reduced to 4 if using 3dp spacer</t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t>CFS25-2</t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">https://item.taobao.com/item.htm?id=639851269279&amp;mi_id=0000hfMFQlFtPVoKWeQYJ5rp5Gr-LZOEgFmY_E5-j2keG-w&amp;spm=a21xtw.29178619.0.0&amp;xxc=shop&amp;skuId=4766125982738 </t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t>Can consider removing if really no money</t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;- not suggested tho</t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
     <t>Coupler</t>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">https://item.taobao.com/item.htm?from=cart&amp;id=567933755449&amp;mi_id=0000khAZDC1_7btHN-U8GeP3VI1kxoi7WNCBXTXU_mOWCw0&amp;skuId=4104578295409&amp;spm=a1z0d.6639537%2F202410.item.d567933755449.3d385886TqyZCj&amp;upStreamPrice=2400 </t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t>MGN9H</t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">https://item.taobao.com/item.htm?abbucket=3&amp;id=1002234653079&amp;mi_id=0000qHfYPQSmfsjcNPJaxefUyUEJRL4Sexc4wRgUKubMZEc&amp;ns=1&amp;priceTId=2100c89317718529411453457e0cdb&amp;skuId=5989891308438&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%2251610e51d45306e6c11e4cc3362f5138%22%7D&amp;xxc=taobaoSearch </t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t>MGN9 Stopper</t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">https://item.taobao.com/item.htm?from=cart&amp;id=712585701882&amp;mi_id=00007mto0iQPp-eh6Ko_hgLbhqYtGV0pkFlIYQMSNlsI7A8&amp;skuId=4988608772418&amp;spm=a1z0d.6639537%2F202410.item.d712585701882.3d3858864s5pmT&amp;upStreamPrice=360 </t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Depends </t>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
@@ -194,10 +142,6 @@
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
-    <t>Borrow? Remove?</t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
     <t>F626ZZ</t>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
@@ -211,10 +155,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://detail.tmall.com/item.htm?abbucket=8&amp;id=683698385971&amp;pisk=gM5jrBg1Pmmjz0zYXmzrA99LMOA1CzPeWVTO-NhqWIdYC5sN4mWV3NnOfNsR_dKNuCa1q3520ZRvfC_hAi-2Qx5SeFTxBch9k4nJVihw31_i1FQOjrxao87coCATYkR_TZb0t4Ow4sMx2bQk7EnYUKhjiah7YkPU1-3J1oZFuDTiTgLBJCLvDdh8Pe8sHCp9kaUWWFovXnIOyztkSch9kjKRyeLwkCLt63HJuEhxXEHx2QKkWCHv6GQ8PF-JXCdOXaHUYuTuhnQb5suYRiZFCZKS6fCYiKtIL3Lkz_ZWHH_AGV0iIE9XvZKuxJZOkLQMC10i1nQAKGYdDmEenNB5VEO_axddPOIBrsFEcUXVyw-RR2hdoI6COIBbqYAVc_dRM9gt6aOXmLLWFmZWvsbRtQpz9y_RZi7cNNuT6USe2Zfv1WUHGIKvNUfaqjK1eOC2nCmYYKbOFgTX9glsTHT9mAgWKfTWYzaSIAAHlwK_gejVxKLkz6z7PmMMHUYWYzaSIAvvrU5UPzijI&amp;rn=706b9c470d1bf18be76c61f71dcf44c0&amp;skuId=5888866023737&amp;spm=a312a.7700824.w4011-25593304449.228.10ec4af44imHfi </t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <t>Maybe don't need to buy if they have stock</t>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
@@ -261,6 +201,13 @@
     <t>Grand Total</t>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?from=cart&amp;id=837011425535&amp;mi_id=00002JJiWREtcmVTrHMfal0z-u4fnfVPven3LmJKz-rVWXQ&amp;skuId=5762086830849&amp;spm=a1z0d.6639537%2F202410.item.d837011425535.45007484wUxzaw&amp;upStreamPrice=1057</t>
+  </si>
+  <si>
+    <t>Trigger button</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -271,7 +218,7 @@
     <numFmt numFmtId="177" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="178" formatCode="_-[$CNY]\ * #,##0.00_-;\-[$CNY]\ * #,##0.00_-;_-[$CNY]\ * &quot;-&quot;??_-;_-@"/>
     <numFmt numFmtId="179" formatCode="_ [$¥-804]* #,##0.00_ ;_ [$¥-804]* \-#,##0.00_ ;_ [$¥-804]* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="180" formatCode="_-[$$-404]* #,##0.00_-;\-[$$-404]* #,##0.00_-;_-[$$-404]* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="181" formatCode="_([$HK$-C04]* #,##0.00_);_([$HK$-C04]* \(#,##0.00\);_([$HK$-C04]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -386,7 +333,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -411,14 +358,8 @@
         <bgColor theme="0"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -579,12 +520,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -648,16 +604,10 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="179" fontId="1" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -669,16 +619,10 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -710,6 +654,57 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -933,10 +928,10 @@
   <dimension ref="A1:U1007"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="1" max="1" width="6.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="86.109375" customWidth="1"/>
-    <col min="4" max="4" width="32.5546875" customWidth="1"/>
+    <col min="3" max="3" width="86.109375" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="32.5546875" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
@@ -948,7 +943,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="19.95" customHeight="1">
-      <c r="A1" s="29"/>
+      <c r="A1" s="26"/>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
@@ -970,29 +965,29 @@
       <c r="T1" s="3"/>
       <c r="U1" s="3"/>
     </row>
-    <row r="2" spans="1:21" ht="31.2" customHeight="1">
-      <c r="A2" s="32" t="s">
+    <row r="2" spans="1:21" ht="31.2">
+      <c r="A2" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="C2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="E2" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="32" t="s">
+      <c r="F2" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="32" t="s">
+      <c r="G2" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="54" t="s">
         <v>7</v>
       </c>
       <c r="I2" s="1"/>
@@ -1009,19 +1004,19 @@
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
     </row>
-    <row r="3" spans="1:21" ht="19.95" customHeight="1">
-      <c r="A3" s="33"/>
-      <c r="B3" s="33"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="33"/>
+    <row r="3" spans="1:21" ht="16.2">
+      <c r="A3" s="29"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="29"/>
       <c r="H3" s="10" t="s">
         <v>8</v>
       </c>
       <c r="I3" s="1"/>
-      <c r="J3" s="27"/>
+      <c r="J3" s="25"/>
       <c r="K3" s="2"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
@@ -1038,10 +1033,10 @@
       <c r="A4" s="11">
         <v>1</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="13"/>
@@ -1059,7 +1054,7 @@
         <v>99</v>
       </c>
       <c r="I4" s="1"/>
-      <c r="J4" s="27"/>
+      <c r="J4" s="25"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
@@ -1076,10 +1071,10 @@
       <c r="A5" s="11">
         <v>2</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="13"/>
@@ -1097,7 +1092,7 @@
         <v>19</v>
       </c>
       <c r="I5" s="4"/>
-      <c r="J5" s="27"/>
+      <c r="J5" s="25"/>
       <c r="K5" s="5"/>
       <c r="L5" s="6"/>
       <c r="M5" s="6"/>
@@ -1114,10 +1109,10 @@
       <c r="A6" s="11">
         <v>3</v>
       </c>
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="21" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="13"/>
@@ -1135,7 +1130,7 @@
         <v>15</v>
       </c>
       <c r="I6" s="1"/>
-      <c r="J6" s="27"/>
+      <c r="J6" s="25"/>
       <c r="K6" s="2"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -1152,10 +1147,10 @@
       <c r="A7" s="11">
         <v>4</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="21" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="13"/>
@@ -1173,7 +1168,7 @@
         <v>22</v>
       </c>
       <c r="I7" s="4"/>
-      <c r="J7" s="27"/>
+      <c r="J7" s="25"/>
       <c r="K7" s="5"/>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
@@ -1190,10 +1185,10 @@
       <c r="A8" s="11">
         <v>5</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="21" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="13"/>
@@ -1211,9 +1206,7 @@
         <v>5.5</v>
       </c>
       <c r="I8" s="7"/>
-      <c r="J8" s="27" t="s">
-        <v>19</v>
-      </c>
+      <c r="J8" s="25"/>
       <c r="K8" s="5"/>
       <c r="L8" s="6"/>
       <c r="M8" s="6"/>
@@ -1230,11 +1223,11 @@
       <c r="A9" s="11">
         <v>6</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="21" t="s">
         <v>20</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>21</v>
       </c>
       <c r="D9" s="13"/>
       <c r="E9" s="14">
@@ -1251,7 +1244,7 @@
         <v>6</v>
       </c>
       <c r="I9" s="9"/>
-      <c r="J9" s="27"/>
+      <c r="J9" s="25"/>
       <c r="K9" s="2"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
@@ -1268,30 +1261,28 @@
       <c r="A10" s="11">
         <v>7</v>
       </c>
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="21" t="s">
         <v>22</v>
-      </c>
-      <c r="C10" s="22" t="s">
-        <v>23</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="14">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F10" s="11" t="s">
         <v>8</v>
       </c>
       <c r="G10" s="15">
-        <v>1.55</v>
+        <v>25</v>
       </c>
       <c r="H10" s="16">
-        <f t="shared" si="0"/>
-        <v>12.4</v>
+        <f>IF(F10 = H$3,$E10*$G10,)</f>
+        <v>75</v>
       </c>
       <c r="I10" s="9"/>
-      <c r="J10" s="27" t="s">
-        <v>24</v>
-      </c>
+      <c r="J10" s="25"/>
       <c r="K10" s="2"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -1308,13 +1299,12 @@
       <c r="A11" s="11">
         <v>8</v>
       </c>
-      <c r="B11" s="31" t="s">
-        <v>25</v>
+      <c r="B11" s="37" t="s">
+        <v>23</v>
       </c>
-      <c r="C11" s="22" t="s">
-        <v>26</v>
+      <c r="C11" s="21" t="s">
+        <v>24</v>
       </c>
-      <c r="D11" s="13"/>
       <c r="E11" s="14">
         <v>1</v>
       </c>
@@ -1322,20 +1312,16 @@
         <v>8</v>
       </c>
       <c r="G11" s="15">
-        <v>40</v>
+        <v>15.8</v>
       </c>
       <c r="H11" s="16">
-        <f t="shared" si="0"/>
-        <v>40</v>
+        <f>IF(F11 = H$3,$E11*$G11,)</f>
+        <v>15.8</v>
       </c>
       <c r="I11" s="9"/>
-      <c r="J11" s="27" t="s">
-        <v>27</v>
-      </c>
+      <c r="J11" s="25"/>
       <c r="K11" s="1"/>
-      <c r="L11" s="27" t="s">
-        <v>28</v>
-      </c>
+      <c r="L11" s="25"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
@@ -1349,28 +1335,27 @@
       <c r="A12" s="11">
         <v>9</v>
       </c>
-      <c r="B12" s="31" t="s">
-        <v>29</v>
+      <c r="B12" s="37" t="s">
+        <v>25</v>
       </c>
-      <c r="C12" s="22" t="s">
-        <v>30</v>
+      <c r="C12" s="21" t="s">
+        <v>26</v>
       </c>
-      <c r="D12" s="13"/>
       <c r="E12" s="14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
         <v>8</v>
       </c>
       <c r="G12" s="15">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="H12" s="16">
-        <f t="shared" si="0"/>
-        <v>75</v>
+        <f>IF(F12 = H$3,$E12*$G12,)</f>
+        <v>68</v>
       </c>
       <c r="I12" s="17"/>
-      <c r="J12" s="27"/>
+      <c r="J12" s="25"/>
       <c r="K12" s="5"/>
       <c r="L12" s="6"/>
       <c r="M12" s="6"/>
@@ -1387,29 +1372,27 @@
       <c r="A13" s="11">
         <v>10</v>
       </c>
-      <c r="B13" s="31" t="s">
-        <v>31</v>
+      <c r="B13" s="37" t="s">
+        <v>27</v>
       </c>
-      <c r="C13" s="22" t="s">
-        <v>32</v>
+      <c r="C13" s="21" t="s">
+        <v>28</v>
       </c>
       <c r="E13" s="14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" s="11" t="s">
         <v>8</v>
       </c>
       <c r="G13" s="15">
-        <v>9</v>
+        <v>2.75</v>
       </c>
       <c r="H13" s="16">
-        <f t="shared" si="0"/>
-        <v>18</v>
+        <f>IF(F13 = H$3,$E13*$G13,)</f>
+        <v>8.25</v>
       </c>
       <c r="I13" s="17"/>
-      <c r="J13" s="27" t="s">
-        <v>19</v>
-      </c>
+      <c r="J13" s="25"/>
       <c r="K13" s="5"/>
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
@@ -1426,29 +1409,27 @@
       <c r="A14" s="11">
         <v>11</v>
       </c>
-      <c r="B14" s="31" t="s">
-        <v>33</v>
+      <c r="B14" s="37" t="s">
+        <v>29</v>
       </c>
-      <c r="C14" s="22" t="s">
-        <v>34</v>
+      <c r="C14" s="21" t="s">
+        <v>30</v>
       </c>
       <c r="E14" s="14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F14" s="11" t="s">
         <v>8</v>
       </c>
       <c r="G14" s="15">
-        <v>4</v>
+        <v>11.18</v>
       </c>
       <c r="H14" s="16">
-        <f t="shared" si="0"/>
-        <v>16</v>
+        <f>IF(F14 = H$3,$E14*$G14,)</f>
+        <v>11.18</v>
       </c>
-      <c r="I14" s="30"/>
-      <c r="J14" s="27" t="s">
-        <v>35</v>
-      </c>
+      <c r="I14" s="27"/>
+      <c r="J14" s="25"/>
       <c r="K14" s="5"/>
       <c r="L14" s="6"/>
       <c r="M14" s="6"/>
@@ -1465,12 +1446,13 @@
       <c r="A15" s="11">
         <v>12</v>
       </c>
-      <c r="B15" s="31" t="s">
-        <v>36</v>
+      <c r="B15" s="37" t="s">
+        <v>31</v>
       </c>
-      <c r="C15" s="22" t="s">
-        <v>37</v>
+      <c r="C15" s="21" t="s">
+        <v>32</v>
       </c>
+      <c r="D15" s="13"/>
       <c r="E15" s="14">
         <v>1</v>
       </c>
@@ -1478,13 +1460,13 @@
         <v>8</v>
       </c>
       <c r="G15" s="15">
-        <v>15.8</v>
+        <v>0</v>
       </c>
       <c r="H15" s="16">
-        <f t="shared" si="0"/>
-        <v>15.8</v>
+        <f>IF(F15 = H$3,$E15*$G15,)</f>
+        <v>0</v>
       </c>
-      <c r="I15" s="30"/>
+      <c r="I15" s="27"/>
       <c r="J15" s="5"/>
       <c r="K15" s="4"/>
       <c r="L15" s="6"/>
@@ -1502,29 +1484,28 @@
       <c r="A16" s="11">
         <v>13</v>
       </c>
-      <c r="B16" s="21" t="s">
-        <v>38</v>
+      <c r="B16" s="37" t="s">
+        <v>33</v>
       </c>
-      <c r="C16" s="22" t="s">
-        <v>39</v>
+      <c r="C16" s="21" t="s">
+        <v>34</v>
       </c>
+      <c r="D16" s="13"/>
       <c r="E16" s="14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F16" s="11" t="s">
         <v>8</v>
       </c>
       <c r="G16" s="15">
-        <v>68</v>
+        <v>13.2</v>
       </c>
       <c r="H16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>IF(F16 = H$3,$E16*$G16,)</f>
+        <v>39.599999999999994</v>
       </c>
       <c r="I16" s="9"/>
-      <c r="J16" s="27" t="s">
-        <v>40</v>
-      </c>
+      <c r="J16" s="25"/>
       <c r="K16" s="5"/>
       <c r="L16" s="6"/>
       <c r="M16" s="6"/>
@@ -1541,24 +1522,25 @@
       <c r="A17" s="11">
         <v>14</v>
       </c>
-      <c r="B17" s="31" t="s">
-        <v>41</v>
+      <c r="B17" s="37" t="s">
+        <v>35</v>
       </c>
-      <c r="C17" s="22" t="s">
-        <v>42</v>
+      <c r="C17" s="21" t="s">
+        <v>36</v>
       </c>
+      <c r="D17" s="13"/>
       <c r="E17" s="14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" s="11" t="s">
         <v>8</v>
       </c>
       <c r="G17" s="15">
-        <v>2.75</v>
+        <v>6.7</v>
       </c>
       <c r="H17" s="16">
-        <f t="shared" si="0"/>
-        <v>8.25</v>
+        <f>IF(F17 = H$3,$E17*$G17,)</f>
+        <v>13.4</v>
       </c>
       <c r="I17" s="9"/>
       <c r="J17" s="4"/>
@@ -1578,12 +1560,13 @@
       <c r="A18" s="11">
         <v>15</v>
       </c>
-      <c r="B18" s="31" t="s">
-        <v>43</v>
+      <c r="B18" s="37" t="s">
+        <v>37</v>
       </c>
-      <c r="C18" s="22" t="s">
-        <v>44</v>
+      <c r="C18" s="21" t="s">
+        <v>38</v>
       </c>
+      <c r="D18" s="13"/>
       <c r="E18" s="14">
         <v>1</v>
       </c>
@@ -1591,16 +1574,14 @@
         <v>8</v>
       </c>
       <c r="G18" s="15">
-        <v>11.18</v>
+        <v>25.65</v>
       </c>
       <c r="H18" s="16">
-        <f t="shared" si="0"/>
-        <v>11.18</v>
+        <f>IF(F18 = H$3,$E18*$G18,)</f>
+        <v>25.65</v>
       </c>
       <c r="I18" s="17"/>
-      <c r="J18" s="27" t="s">
-        <v>45</v>
-      </c>
+      <c r="J18" s="25"/>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
@@ -1617,25 +1598,25 @@
       <c r="A19" s="11">
         <v>16</v>
       </c>
-      <c r="B19" s="21" t="s">
-        <v>46</v>
+      <c r="B19" s="37" t="s">
+        <v>39</v>
       </c>
-      <c r="C19" s="22" t="s">
-        <v>47</v>
+      <c r="C19" s="21" t="s">
+        <v>40</v>
       </c>
       <c r="D19" s="13"/>
       <c r="E19" s="14">
         <v>1</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="G19" s="15">
-        <v>0</v>
+      <c r="G19" s="24">
+        <v>10.56</v>
       </c>
       <c r="H19" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>IF(F19 = H$3,$E19*$G19,)</f>
+        <v>10.56</v>
       </c>
       <c r="I19" s="17"/>
       <c r="J19" s="4"/>
@@ -1652,30 +1633,30 @@
       <c r="U19" s="6"/>
     </row>
     <row r="20" spans="1:21" ht="19.95" customHeight="1">
-      <c r="A20" s="11">
+      <c r="A20" s="47">
         <v>17</v>
       </c>
-      <c r="B20" s="31" t="s">
-        <v>48</v>
+      <c r="B20" s="48" t="s">
+        <v>43</v>
       </c>
-      <c r="C20" s="22" t="s">
-        <v>49</v>
+      <c r="C20" s="49" t="s">
+        <v>42</v>
       </c>
-      <c r="D20" s="13"/>
-      <c r="E20" s="14">
-        <v>3</v>
+      <c r="D20" s="50"/>
+      <c r="E20" s="51">
+        <v>1</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="G20" s="15">
-        <v>13.2</v>
+      <c r="G20" s="52">
+        <v>1.5</v>
       </c>
-      <c r="H20" s="16">
-        <f t="shared" si="0"/>
-        <v>39.599999999999994</v>
+      <c r="H20" s="53">
+        <f>IF(F20 = H$3,$E20*$G20,)</f>
+        <v>1.5</v>
       </c>
-      <c r="I20" s="30"/>
+      <c r="I20" s="27"/>
       <c r="J20" s="4"/>
       <c r="K20" s="5"/>
       <c r="L20" s="6"/>
@@ -1690,30 +1671,20 @@
       <c r="U20" s="6"/>
     </row>
     <row r="21" spans="1:21" ht="19.95" customHeight="1">
-      <c r="A21" s="11">
-        <v>18</v>
+      <c r="A21" s="41"/>
+      <c r="B21" s="41"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="32" t="s">
+        <v>41</v>
       </c>
-      <c r="B21" s="31" t="s">
-        <v>50</v>
+      <c r="G21" s="33"/>
+      <c r="H21" s="22">
+        <f>SUM(H4:H20)</f>
+        <v>435.44</v>
       </c>
-      <c r="C21" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" s="13"/>
-      <c r="E21" s="14">
-        <v>2</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="G21" s="15">
-        <v>6.7</v>
-      </c>
-      <c r="H21" s="16">
-        <f t="shared" si="0"/>
-        <v>13.4</v>
-      </c>
-      <c r="I21" s="9"/>
+      <c r="I21" s="38"/>
       <c r="J21" s="4"/>
       <c r="K21" s="5"/>
       <c r="L21" s="6"/>
@@ -1728,30 +1699,18 @@
       <c r="U21" s="6"/>
     </row>
     <row r="22" spans="1:21" ht="19.95" customHeight="1">
-      <c r="A22" s="11">
-        <v>19</v>
+      <c r="A22" s="42"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="44"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="35"/>
+      <c r="H22" s="40">
+        <f>H21*1.15</f>
+        <v>500.75599999999997</v>
       </c>
-      <c r="B22" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>53</v>
-      </c>
-      <c r="D22" s="13"/>
-      <c r="E22" s="14">
-        <v>1</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="G22" s="15">
-        <v>25.65</v>
-      </c>
-      <c r="H22" s="16">
-        <f t="shared" si="0"/>
-        <v>25.65</v>
-      </c>
-      <c r="I22" s="9"/>
+      <c r="I22" s="38"/>
       <c r="J22" s="1"/>
       <c r="K22" s="2"/>
       <c r="L22" s="1"/>
@@ -1766,30 +1725,7 @@
       <c r="U22" s="1"/>
     </row>
     <row r="23" spans="1:21" ht="19.95" customHeight="1">
-      <c r="A23" s="11">
-        <v>20</v>
-      </c>
-      <c r="B23" s="31" t="s">
-        <v>54</v>
-      </c>
-      <c r="C23" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="14">
-        <v>1</v>
-      </c>
-      <c r="F23" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="G23" s="26">
-        <v>10.56</v>
-      </c>
-      <c r="H23" s="16">
-        <f t="shared" si="0"/>
-        <v>10.56</v>
-      </c>
-      <c r="I23" s="9"/>
+      <c r="I23" s="38"/>
       <c r="J23" s="1"/>
       <c r="K23" s="2"/>
       <c r="L23" s="1"/>
@@ -1804,20 +1740,7 @@
       <c r="U23" s="1"/>
     </row>
     <row r="24" spans="1:21" ht="19.95" customHeight="1">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="G24" s="37"/>
-      <c r="H24" s="23">
-        <f>SUM(H4:H23)</f>
-        <v>452.34</v>
-      </c>
-      <c r="I24" s="17"/>
+      <c r="I24" s="39"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
@@ -1832,18 +1755,7 @@
       <c r="U24" s="1"/>
     </row>
     <row r="25" spans="1:21" ht="19.95" customHeight="1">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="39"/>
-      <c r="H25" s="24">
-        <f>H24*1.13</f>
-        <v>511.1441999999999</v>
-      </c>
-      <c r="I25" s="17"/>
+      <c r="I25" s="39"/>
       <c r="J25" s="1"/>
       <c r="K25" s="5"/>
       <c r="L25" s="6"/>
@@ -1884,9 +1796,6 @@
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
       <c r="I27" s="6"/>
       <c r="J27" s="6"/>
       <c r="K27" s="5"/>
@@ -1907,9 +1816,6 @@
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="5"/>
@@ -24439,7 +24345,7 @@
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
-    <mergeCell ref="F24:G25"/>
+    <mergeCell ref="F21:G22"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:F3"/>
@@ -24447,7 +24353,7 @@
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F52 F4:F23 F27:F34" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F52 F4:F22 F29:F34" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$H$3:$H$3</formula1>
     </dataValidation>
   </dataValidations>
@@ -24456,18 +24362,15 @@
     <hyperlink ref="C6" r:id="rId2" xr:uid="{FC44491B-FDFC-4021-8651-E19D9223C216}"/>
     <hyperlink ref="C7" r:id="rId3" xr:uid="{350EF2DA-9D2B-404F-A5EC-0413DB3D5B8A}"/>
     <hyperlink ref="C8" r:id="rId4" xr:uid="{56356BE3-485A-455B-A6AD-0EB2C60F3B81}"/>
-    <hyperlink ref="C10" r:id="rId5" xr:uid="{85E12540-2EA9-43F6-B909-BA97D126881B}"/>
-    <hyperlink ref="C11" r:id="rId6" xr:uid="{A9B6F69C-0B33-415C-A3AB-A69BB734A8B1}"/>
-    <hyperlink ref="C12" r:id="rId7" xr:uid="{AC7B88C6-5615-44F2-808E-EF62AF1290E0}"/>
-    <hyperlink ref="C13" r:id="rId8" display="https://item.taobao.com/item.htm?abbucket=3&amp;id=1002234653079&amp;mi_id=0000qHfYPQSmfsjcNPJaxefUyUEJRL4Sexc4wRgUKubMZEc&amp;ns=1&amp;priceTId=2100c89317718529411453457e0cdb&amp;skuId=5989891308438&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%2251610e51d45306e6c11e4cc3362f5138%22%7D&amp;xxc=taobaoSearch " xr:uid="{B98A09AE-03E9-4114-95FC-44D8D1C16634}"/>
-    <hyperlink ref="C14" r:id="rId9" xr:uid="{5DA2E89D-FDC8-4695-BE44-011F8B0D81BB}"/>
-    <hyperlink ref="C16" r:id="rId10" display="https://item.taobao.com/item.htm?abbucket=3&amp;id=773044688198&amp;mi_id=0000o0TQRHP5WYfrXn7yVnNYE7hnSj8OjiIN9DrkrLe5zTw&amp;ns=1&amp;priceTId=2100c89317718532634203533e0cdb&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%22f302a93986c91eb5bf3d5fda48988bfd%22%7D&amp;xxc=taobaoSearch&amp;skuId=5463603075088 " xr:uid="{C5566206-30D7-4F34-A888-74FA7C8787C1}"/>
-    <hyperlink ref="C17" r:id="rId11" display="https://item.taobao.com/item.htm?abbucket=3&amp;id=787710083854&amp;mi_id=0000dH7WFqPo0VTsYjpnAS_Q4XCGEMyEbrfLht3nhTk_3H4&amp;ns=1&amp;priceTId=2100c89317718533692436712e0cdb&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%224c2fa0c1d9d46ededc0a99b18837d993%22%7D&amp;xxc=taobaoSearch&amp;skuId=5548210563574 " xr:uid="{5690B020-D1A3-4339-8042-2162A97F3CB0}"/>
-    <hyperlink ref="C23" r:id="rId12" xr:uid="{0484DBBF-F685-48B0-905A-A2B15A604B44}"/>
-    <hyperlink ref="C15" r:id="rId13" display="https://item.taobao.com/item.htm?abbucket=3&amp;id=588096657853&amp;mi_id=0000wcrxEWxjGnVqV1EtPKLfYc-xaoayPOO1ndrYif0qneY&amp;ns=1&amp;priceTId=2100c89317718531649681067e0cdb&amp;skuId=4009433069850&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%22a8937da123f65f19e1c9c155c626044f%22%7D&amp;xxc=taobaoSearch " xr:uid="{80D3A539-58C2-424B-8BD2-310D221BB87D}"/>
-    <hyperlink ref="C21" r:id="rId14" xr:uid="{B8FB3FF0-079E-4D70-A34D-786B50399894}"/>
-    <hyperlink ref="C22" r:id="rId15" xr:uid="{D2604814-835B-43C3-93C4-9E68179BCB52}"/>
-    <hyperlink ref="C4" r:id="rId16" xr:uid="{8ABEDF76-66B2-442D-A4B1-E2728F99D099}"/>
+    <hyperlink ref="C10" r:id="rId5" xr:uid="{AC7B88C6-5615-44F2-808E-EF62AF1290E0}"/>
+    <hyperlink ref="C12" r:id="rId6" display="https://item.taobao.com/item.htm?abbucket=3&amp;id=773044688198&amp;mi_id=0000o0TQRHP5WYfrXn7yVnNYE7hnSj8OjiIN9DrkrLe5zTw&amp;ns=1&amp;priceTId=2100c89317718532634203533e0cdb&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%22f302a93986c91eb5bf3d5fda48988bfd%22%7D&amp;xxc=taobaoSearch&amp;skuId=5463603075088 " xr:uid="{C5566206-30D7-4F34-A888-74FA7C8787C1}"/>
+    <hyperlink ref="C13" r:id="rId7" display="https://item.taobao.com/item.htm?abbucket=3&amp;id=787710083854&amp;mi_id=0000dH7WFqPo0VTsYjpnAS_Q4XCGEMyEbrfLht3nhTk_3H4&amp;ns=1&amp;priceTId=2100c89317718533692436712e0cdb&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%224c2fa0c1d9d46ededc0a99b18837d993%22%7D&amp;xxc=taobaoSearch&amp;skuId=5548210563574 " xr:uid="{5690B020-D1A3-4339-8042-2162A97F3CB0}"/>
+    <hyperlink ref="C19" r:id="rId8" xr:uid="{0484DBBF-F685-48B0-905A-A2B15A604B44}"/>
+    <hyperlink ref="C11" r:id="rId9" display="https://item.taobao.com/item.htm?abbucket=3&amp;id=588096657853&amp;mi_id=0000wcrxEWxjGnVqV1EtPKLfYc-xaoayPOO1ndrYif0qneY&amp;ns=1&amp;priceTId=2100c89317718531649681067e0cdb&amp;skuId=4009433069850&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%22a8937da123f65f19e1c9c155c626044f%22%7D&amp;xxc=taobaoSearch " xr:uid="{80D3A539-58C2-424B-8BD2-310D221BB87D}"/>
+    <hyperlink ref="C17" r:id="rId10" xr:uid="{B8FB3FF0-079E-4D70-A34D-786B50399894}"/>
+    <hyperlink ref="C18" r:id="rId11" xr:uid="{D2604814-835B-43C3-93C4-9E68179BCB52}"/>
+    <hyperlink ref="C4" r:id="rId12" xr:uid="{8ABEDF76-66B2-442D-A4B1-E2728F99D099}"/>
+    <hyperlink ref="C20" r:id="rId13" display="https://item.taobao.com/item.htm?from=cart&amp;id=837011425535&amp;mi_id=00002JJiWREtcmVTrHMfal0z-u4fnfVPven3LmJKz-rVWXQ&amp;skuId=5762086830849&amp;spm=a1z0d.6639537%2F202410.item.d837011425535.45007484wUxzaw&amp;upStreamPrice=1056 " xr:uid="{38F670C9-E9DE-4617-8757-13A3F1203E06}"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>